<commit_message>
Formatted Row Height, Column Height, Title Bar as a Data Table
</commit_message>
<xml_diff>
--- a/Day 4/Data Cleaning Start.xlsx
+++ b/Day 4/Data Cleaning Start.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2142E954-0143-427B-8BCE-57BDF6FB0F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA16C714-54BF-4BFA-B5F9-EDB2B60F850D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{7F7E1DDE-3781-814A-825E-072C922D74F6}"/>
   </bookViews>
@@ -262,7 +262,7 @@
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -277,16 +277,37 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -294,21 +315,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="6" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -628,862 +674,867 @@
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.69921875" customWidth="1"/>
-    <col min="2" max="2" width="7.19921875" customWidth="1"/>
-    <col min="3" max="3" width="11" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="6.69921875" customWidth="1"/>
-    <col min="9" max="9" width="5.5" customWidth="1"/>
+    <col min="2" max="2" width="12.5" customWidth="1"/>
+    <col min="3" max="3" width="47.69921875" customWidth="1"/>
+    <col min="4" max="4" width="20.09765625" customWidth="1"/>
+    <col min="5" max="5" width="21.296875" customWidth="1"/>
+    <col min="6" max="6" width="10.796875" customWidth="1"/>
+    <col min="7" max="7" width="11.3984375" customWidth="1"/>
+    <col min="8" max="8" width="12.59765625" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
+    <row r="2" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B3" s="4">
+    <row r="3" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B3" s="3">
         <v>45076</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="4">
         <v>4500</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="4">
         <v>598</v>
       </c>
-      <c r="I3" s="2">
+      <c r="I3" s="5">
         <f>H3/G3</f>
         <v>0.13288888888888889</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B4" s="4">
+    <row r="4" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B4" s="3">
         <v>45076</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="4">
         <v>3800</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="4">
         <v>1045</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="5">
         <f t="shared" ref="I4:I32" si="0">H4/G4</f>
         <v>0.27500000000000002</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B5" s="4">
+    <row r="5" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B5" s="3">
         <v>45076</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="1">
+      <c r="F5" s="2"/>
+      <c r="G5" s="4">
         <v>3712.5</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="4">
         <v>1009</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="5">
         <f t="shared" si="0"/>
         <v>0.2717845117845118</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B6" s="4">
+    <row r="6" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B6" s="3">
         <v>45076</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1">
+      <c r="F6" s="2"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4">
         <v>779</v>
       </c>
-      <c r="I6" s="2" t="e">
+      <c r="I6" s="5" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B7" s="4">
+    <row r="7" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B7" s="3">
         <v>45076</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7" s="4">
         <v>5000</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="4">
         <v>684</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="5">
         <f t="shared" si="0"/>
         <v>0.1368</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="4">
+    <row r="8" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B8" s="3">
         <v>45077</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8" s="4">
         <v>6100</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="4">
         <v>544</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="5">
         <f t="shared" si="0"/>
         <v>8.9180327868852466E-2</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B9" s="4">
+    <row r="9" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B9" s="3">
         <v>45077</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9" s="4">
         <v>4625</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="4">
         <v>670</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="5">
         <f t="shared" si="0"/>
         <v>0.14486486486486486</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B10" s="4">
+    <row r="10" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B10" s="3">
         <v>45077</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10" s="4">
         <v>3800</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="4">
         <v>2045</v>
       </c>
-      <c r="I10" s="2">
+      <c r="I10" s="5">
         <f t="shared" si="0"/>
         <v>0.53815789473684206</v>
       </c>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B11" s="4">
+    <row r="11" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B11" s="3">
         <v>45077</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11" s="4">
         <v>3600</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="4">
         <v>1564</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I11" s="5">
         <f t="shared" si="0"/>
         <v>0.43444444444444447</v>
       </c>
     </row>
-    <row r="12" spans="2:9" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="4">
+    <row r="12" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B12" s="3">
         <v>45077</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="4">
         <v>5100</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="4">
         <v>1220</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="5">
         <f t="shared" si="0"/>
         <v>0.23921568627450981</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B13" s="4">
+    <row r="13" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B13" s="3">
         <v>45077</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="4">
         <v>4750</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="4">
         <v>1435</v>
       </c>
-      <c r="I13" s="2">
+      <c r="I13" s="5">
         <f t="shared" si="0"/>
         <v>0.30210526315789471</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B14" s="4">
+    <row r="14" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B14" s="3">
         <v>45077</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="4">
         <v>6000</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="4">
         <v>998</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="5">
         <f t="shared" si="0"/>
         <v>0.16633333333333333</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B15" s="4">
+    <row r="15" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B15" s="3">
         <v>45077</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G15" s="1">
+      <c r="G15" s="4">
         <v>4500</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="4">
         <v>780</v>
       </c>
-      <c r="I15" s="2">
+      <c r="I15" s="5">
         <f t="shared" si="0"/>
         <v>0.17333333333333334</v>
       </c>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B16" s="4">
+    <row r="16" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B16" s="3">
         <v>45078</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1">
+      <c r="G16" s="4"/>
+      <c r="H16" s="4">
         <v>1044</v>
       </c>
-      <c r="I16" s="2" t="e">
+      <c r="I16" s="5" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B17" s="4">
+    <row r="17" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B17" s="3">
         <v>45078</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G17" s="1">
+      <c r="G17" s="4">
         <v>3712.5</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="4">
         <v>1222</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="5">
         <f t="shared" si="0"/>
         <v>0.32915824915824915</v>
       </c>
     </row>
-    <row r="18" spans="2:9" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="4">
+    <row r="18" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B18" s="3">
         <v>45078</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G18" s="1">
+      <c r="G18" s="4">
         <v>4950</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="4">
         <v>1065</v>
       </c>
-      <c r="I18" s="2">
+      <c r="I18" s="5">
         <f t="shared" si="0"/>
         <v>0.21515151515151515</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B19" s="4">
+    <row r="19" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B19" s="3">
         <v>45078</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G19" s="1">
+      <c r="G19" s="4">
         <v>4750</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="4">
         <v>810</v>
       </c>
-      <c r="I19" s="2">
+      <c r="I19" s="5">
         <f t="shared" si="0"/>
         <v>0.17052631578947369</v>
       </c>
     </row>
-    <row r="20" spans="2:9" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="4">
+    <row r="20" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B20" s="3">
         <v>45078</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G20" s="1">
+      <c r="G20" s="4">
         <v>7320</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="4">
         <v>933</v>
       </c>
-      <c r="I20" s="2">
+      <c r="I20" s="5">
         <f t="shared" si="0"/>
         <v>0.12745901639344262</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B21" s="4">
+    <row r="21" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B21" s="3">
         <v>45077</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G21" s="1">
+      <c r="G21" s="4">
         <v>6000</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="4">
         <v>998</v>
       </c>
-      <c r="I21" s="2">
+      <c r="I21" s="5">
         <f t="shared" ref="I21:I22" si="1">H21/G21</f>
         <v>0.16633333333333333</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B22" s="4">
+    <row r="22" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B22" s="3">
         <v>45077</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G22" s="1">
+      <c r="G22" s="4">
         <v>4500</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="4">
         <v>780</v>
       </c>
-      <c r="I22" s="2">
+      <c r="I22" s="5">
         <f t="shared" si="1"/>
         <v>0.17333333333333334</v>
       </c>
     </row>
-    <row r="23" spans="2:9" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="4">
+    <row r="23" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B23" s="3">
         <v>45078</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G23" s="1">
+      <c r="G23" s="4">
         <v>5087.5</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="4">
         <v>655</v>
       </c>
-      <c r="I23" s="2">
+      <c r="I23" s="5">
         <f t="shared" si="0"/>
         <v>0.12874692874692875</v>
       </c>
     </row>
-    <row r="24" spans="2:9" ht="96" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="4">
+    <row r="24" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B24" s="3">
         <v>45078</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G24" s="1">
+      <c r="G24" s="4">
         <v>4500</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="4">
         <v>722</v>
       </c>
-      <c r="I24" s="2">
+      <c r="I24" s="5">
         <f t="shared" si="0"/>
         <v>0.16044444444444445</v>
       </c>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B25" s="4">
+    <row r="25" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B25" s="3">
         <v>45078</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G25" s="1">
+      <c r="G25" s="4">
         <v>4250</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="4">
         <v>901</v>
       </c>
-      <c r="I25" s="2">
+      <c r="I25" s="5">
         <f t="shared" si="0"/>
         <v>0.21199999999999999</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B26" s="4">
+    <row r="26" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B26" s="3">
         <v>45079</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="G26" s="1">
+      <c r="G26" s="4">
         <v>5250</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="4">
         <v>1349</v>
       </c>
-      <c r="I26" s="2">
+      <c r="I26" s="5">
         <f t="shared" si="0"/>
         <v>0.25695238095238093</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B27" s="4">
+    <row r="27" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B27" s="3">
         <v>45079</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="G27" s="1">
+      <c r="G27" s="4">
         <v>6500</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="4">
         <v>1288</v>
       </c>
-      <c r="I27" s="2">
+      <c r="I27" s="5">
         <f t="shared" si="0"/>
         <v>0.19815384615384615</v>
       </c>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B28" s="4">
+    <row r="28" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B28" s="3">
         <v>45079</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F28" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="G28" s="1">
+      <c r="G28" s="4">
         <v>7500</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="4">
         <v>1664</v>
       </c>
-      <c r="I28" s="2">
+      <c r="I28" s="5">
         <f t="shared" si="0"/>
         <v>0.22186666666666666</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B29" s="4">
+    <row r="29" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B29" s="3">
         <v>45079</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G29" s="1">
+      <c r="G29" s="4">
         <v>5500</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="4">
         <v>1320</v>
       </c>
-      <c r="I29" s="2">
+      <c r="I29" s="5">
         <f t="shared" si="0"/>
         <v>0.24</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B30" s="4">
+    <row r="30" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B30" s="3">
         <v>45079</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G30" s="1">
+      <c r="G30" s="4">
         <v>4625</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="4">
         <v>1001</v>
       </c>
-      <c r="I30" s="2">
+      <c r="I30" s="5">
         <f t="shared" si="0"/>
         <v>0.21643243243243243</v>
       </c>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B31" s="4">
+    <row r="31" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B31" s="3">
         <v>45079</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F31" t="s">
+      <c r="F31" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G31" s="1">
+      <c r="G31" s="4">
         <v>4500</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="4">
         <v>960</v>
       </c>
-      <c r="I31" s="2">
+      <c r="I31" s="5">
         <f t="shared" si="0"/>
         <v>0.21333333333333335</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B32" s="4">
+    <row r="32" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B32" s="3">
         <v>45079</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G32" s="1">
+      <c r="G32" s="4">
         <v>5400</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="4">
         <v>540</v>
       </c>
-      <c r="I32" s="2">
+      <c r="I32" s="5">
         <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B33" s="4">
+    <row r="33" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+      <c r="B33" s="3">
         <v>45076</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G33" s="1">
+      <c r="G33" s="4">
         <v>5000</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="4">
         <v>684</v>
       </c>
-      <c r="I33" s="2">
+      <c r="I33" s="5">
         <f t="shared" ref="I33" si="2">H33/G33</f>
         <v>0.1368</v>
       </c>
@@ -1517,5 +1568,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Removed Extra text within bracket beside Clients and make Client name to lower case
</commit_message>
<xml_diff>
--- a/Day 4/Data Cleaning Start.xlsx
+++ b/Day 4/Data Cleaning Start.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C2756EE-5BA7-4C38-84AB-1BFE5AA17AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CABC14A0-289A-4A27-A049-270310B7F492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{7F7E1DDE-3781-814A-825E-072C922D74F6}"/>
   </bookViews>
@@ -169,88 +169,88 @@
     <t>Big Data_California</t>
   </si>
   <si>
-    <t xml:space="preserve">AMAZON.COM, INC. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">TESLA, INC. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">NETFLIX, INC. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">THE PROCTER &amp; GAMBLE COMPANY </t>
-  </si>
-  <si>
-    <t xml:space="preserve">THE GOLDMAN SACHS GROUP, INC. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">JPMORGAN CHASE &amp; CO. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MORGAN STANLEY </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CITIGROUP INC. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BANK OF AMERICA CORPORATION </t>
-  </si>
-  <si>
-    <t xml:space="preserve">WALMART INC. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">TARGET CORPORATION </t>
-  </si>
-  <si>
-    <t xml:space="preserve">COSTCO WHOLESALE CORPORATION </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCDONALD'S CORPORATION </t>
-  </si>
-  <si>
-    <t xml:space="preserve">EXXON MOBIL CORPORATION </t>
-  </si>
-  <si>
-    <t xml:space="preserve">VERIZON COMMUNICATIONS INC. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">THE HOME DEPOT, INC. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CISCO SYSTEMS, INC. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHEVRON CORPORATION </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AT&amp;T INC. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">INTEL CORPORATION </t>
-  </si>
-  <si>
-    <t xml:space="preserve">GENERAL MOTORS COMPANY </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MICROSOFT CORPORATION </t>
-  </si>
-  <si>
-    <t xml:space="preserve">COMCAST CORPORATION </t>
-  </si>
-  <si>
-    <t xml:space="preserve">DELL TECHNOLOGIES INC. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">JOHNSON &amp; JOHNSON </t>
-  </si>
-  <si>
-    <t xml:space="preserve">FEDEX CORPORATION </t>
-  </si>
-  <si>
-    <t xml:space="preserve">GENERAL ELECTRIC COMPANY </t>
-  </si>
-  <si>
-    <t xml:space="preserve">LOCKHEED MARTIN CORPORATION </t>
+    <t xml:space="preserve">amazon.com, inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">tesla, inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">netflix, inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">the procter &amp; gamble company </t>
+  </si>
+  <si>
+    <t xml:space="preserve">the goldman sachs group, inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">jpmorgan chase &amp; co. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">morgan stanley </t>
+  </si>
+  <si>
+    <t xml:space="preserve">citigroup inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">bank of america corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">walmart inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">target corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">costco wholesale corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">mcdonald's corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">exxon mobil corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">verizon communications inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">the home depot, inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cisco systems, inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">chevron corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">at&amp;t inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">intel corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">general motors company </t>
+  </si>
+  <si>
+    <t xml:space="preserve">microsoft corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">comcast corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">dell technologies inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">johnson &amp; johnson </t>
+  </si>
+  <si>
+    <t xml:space="preserve">fedex corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">general electric company </t>
+  </si>
+  <si>
+    <t xml:space="preserve">lockheed martin corporation </t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Contact names are trimmed and fixed using trim and proper function
</commit_message>
<xml_diff>
--- a/Day 4/Data Cleaning Start.xlsx
+++ b/Day 4/Data Cleaning Start.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CABC14A0-289A-4A27-A049-270310B7F492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB34289A-6247-4803-90FF-AD7469076961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{7F7E1DDE-3781-814A-825E-072C922D74F6}"/>
   </bookViews>
@@ -73,27 +73,6 @@
     <t>Mik Naam</t>
   </si>
   <si>
-    <t xml:space="preserve">     Bill SmITH</t>
-  </si>
-  <si>
-    <t>KEN Singh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Harley        Fritz</t>
-  </si>
-  <si>
-    <t>David    Rasmussen</t>
-  </si>
-  <si>
-    <t>IVAN HINEY</t>
-  </si>
-  <si>
-    <t>JONha Ma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     Jordan Boone</t>
-  </si>
-  <si>
     <t>Payment</t>
   </si>
   <si>
@@ -109,54 +88,6 @@
     <t>Transfer</t>
   </si>
   <si>
-    <t>BRENDAN Wallace</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     Conor Wise</t>
-  </si>
-  <si>
-    <t>Steven     MIChael</t>
-  </si>
-  <si>
-    <t>JoSE   Roach</t>
-  </si>
-  <si>
-    <t>Franklin WRIGT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Alia       Thornton</t>
-  </si>
-  <si>
-    <t>Denzel        Flores</t>
-  </si>
-  <si>
-    <t>Bruno CordOVA</t>
-  </si>
-  <si>
-    <t>jaylynn   napp</t>
-  </si>
-  <si>
-    <t>Bruce RICH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     Arturo Moore</t>
-  </si>
-  <si>
-    <t>Bryce     Carpenter</t>
-  </si>
-  <si>
-    <t>Jaidyn ANDERSEN</t>
-  </si>
-  <si>
-    <t>MARK WALM</t>
-  </si>
-  <si>
-    <t>HARRY LEE</t>
-  </si>
-  <si>
-    <t>JOSH JOHNSON</t>
-  </si>
-  <si>
     <t>Cloud Tech_Texas</t>
   </si>
   <si>
@@ -251,6 +182,75 @@
   </si>
   <si>
     <t xml:space="preserve">lockheed martin corporation </t>
+  </si>
+  <si>
+    <t>Bill Smith</t>
+  </si>
+  <si>
+    <t>Ken Singh</t>
+  </si>
+  <si>
+    <t>Harley Fritz</t>
+  </si>
+  <si>
+    <t>David Rasmussen</t>
+  </si>
+  <si>
+    <t>Ivan Hiney</t>
+  </si>
+  <si>
+    <t>Jonha Ma</t>
+  </si>
+  <si>
+    <t>Jordan Boone</t>
+  </si>
+  <si>
+    <t>Brendan Wallace</t>
+  </si>
+  <si>
+    <t>Conor Wise</t>
+  </si>
+  <si>
+    <t>Steven Michael</t>
+  </si>
+  <si>
+    <t>Jose Roach</t>
+  </si>
+  <si>
+    <t>Franklin Wrigt</t>
+  </si>
+  <si>
+    <t>Alia Thornton</t>
+  </si>
+  <si>
+    <t>Denzel Flores</t>
+  </si>
+  <si>
+    <t>Bruno Cordova</t>
+  </si>
+  <si>
+    <t>Jaylynn Napp</t>
+  </si>
+  <si>
+    <t>Bruce Rich</t>
+  </si>
+  <si>
+    <t>Arturo Moore</t>
+  </si>
+  <si>
+    <t>Bryce Carpenter</t>
+  </si>
+  <si>
+    <t>Jaidyn Andersen</t>
+  </si>
+  <si>
+    <t>Mark Walm</t>
+  </si>
+  <si>
+    <t>Harry Lee</t>
+  </si>
+  <si>
+    <t>Josh Johnson</t>
   </si>
 </sst>
 </file>
@@ -697,7 +697,7 @@
         <v>6</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>2</v>
@@ -714,16 +714,16 @@
         <v>45076</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G3" s="4">
         <v>4500</v>
@@ -741,16 +741,16 @@
         <v>45076</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G4" s="4">
         <v>3800</v>
@@ -768,13 +768,13 @@
         <v>45076</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="4">
@@ -793,13 +793,13 @@
         <v>45076</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="4"/>
@@ -816,16 +816,16 @@
         <v>45076</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="G7" s="4">
         <v>5000</v>
@@ -843,16 +843,16 @@
         <v>45077</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="G8" s="4">
         <v>6100</v>
@@ -870,16 +870,16 @@
         <v>45077</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="F9" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G9" s="4">
         <v>4625</v>
@@ -897,16 +897,16 @@
         <v>45077</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G10" s="4">
         <v>3800</v>
@@ -924,16 +924,16 @@
         <v>45077</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G11" s="4">
         <v>3600</v>
@@ -951,16 +951,16 @@
         <v>45077</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="G12" s="4">
         <v>5100</v>
@@ -978,16 +978,16 @@
         <v>45077</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="G13" s="4">
         <v>4750</v>
@@ -1005,16 +1005,16 @@
         <v>45077</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G14" s="4">
         <v>6000</v>
@@ -1032,16 +1032,16 @@
         <v>45077</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="G15" s="4">
         <v>4500</v>
@@ -1059,16 +1059,16 @@
         <v>45078</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4">
@@ -1084,16 +1084,16 @@
         <v>45078</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G17" s="4">
         <v>3712.5</v>
@@ -1111,16 +1111,16 @@
         <v>45078</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G18" s="4">
         <v>4950</v>
@@ -1138,16 +1138,16 @@
         <v>45078</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G19" s="4">
         <v>4750</v>
@@ -1165,16 +1165,16 @@
         <v>45078</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G20" s="4">
         <v>7320</v>
@@ -1192,16 +1192,16 @@
         <v>45077</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G21" s="4">
         <v>6000</v>
@@ -1219,16 +1219,16 @@
         <v>45077</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="G22" s="4">
         <v>4500</v>
@@ -1246,16 +1246,16 @@
         <v>45078</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>31</v>
+        <v>63</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G23" s="4">
         <v>5087.5</v>
@@ -1273,16 +1273,16 @@
         <v>45078</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G24" s="4">
         <v>4500</v>
@@ -1300,16 +1300,16 @@
         <v>45078</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G25" s="4">
         <v>4250</v>
@@ -1327,16 +1327,16 @@
         <v>45079</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>34</v>
+        <v>66</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G26" s="4">
         <v>5250</v>
@@ -1354,16 +1354,16 @@
         <v>45079</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G27" s="4">
         <v>6500</v>
@@ -1381,16 +1381,16 @@
         <v>45079</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G28" s="4">
         <v>7500</v>
@@ -1408,16 +1408,16 @@
         <v>45079</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>37</v>
+        <v>69</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G29" s="4">
         <v>5500</v>
@@ -1435,16 +1435,16 @@
         <v>45079</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>38</v>
+        <v>70</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G30" s="4">
         <v>4625</v>
@@ -1462,16 +1462,16 @@
         <v>45079</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G31" s="4">
         <v>4500</v>
@@ -1489,16 +1489,16 @@
         <v>45079</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G32" s="4">
         <v>5400</v>
@@ -1516,16 +1516,16 @@
         <v>45076</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="D33" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="G33" s="4">
         <v>5000</v>

</xml_diff>

<commit_message>
State name is separated from the Department text using Text to Columns
</commit_message>
<xml_diff>
--- a/Day 4/Data Cleaning Start.xlsx
+++ b/Day 4/Data Cleaning Start.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB34289A-6247-4803-90FF-AD7469076961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20058B7-D13C-41CD-9028-CE77F77F9C90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{7F7E1DDE-3781-814A-825E-072C922D74F6}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="77">
   <si>
     <t>Date</t>
   </si>
@@ -88,18 +88,6 @@
     <t>Transfer</t>
   </si>
   <si>
-    <t>Cloud Tech_Texas</t>
-  </si>
-  <si>
-    <t>Strategy_New York</t>
-  </si>
-  <si>
-    <t>Operations_Florida</t>
-  </si>
-  <si>
-    <t>Big Data_California</t>
-  </si>
-  <si>
     <t xml:space="preserve">amazon.com, inc. </t>
   </si>
   <si>
@@ -251,6 +239,33 @@
   </si>
   <si>
     <t>Josh Johnson</t>
+  </si>
+  <si>
+    <t>Cloud Tech</t>
+  </si>
+  <si>
+    <t>Texas</t>
+  </si>
+  <si>
+    <t>Strategy</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>Operations</t>
+  </si>
+  <si>
+    <t>Florida</t>
+  </si>
+  <si>
+    <t>Big Data</t>
+  </si>
+  <si>
+    <t>California</t>
+  </si>
+  <si>
+    <t>State</t>
   </si>
 </sst>
 </file>
@@ -669,21 +684,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD37A31F-92F2-FA4A-B7ED-0F04A433817B}">
-  <dimension ref="B2:I42"/>
+  <dimension ref="B2:J42"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.69921875" customWidth="1"/>
     <col min="2" max="2" width="12.5" customWidth="1"/>
     <col min="3" max="3" width="47.69921875" customWidth="1"/>
     <col min="4" max="4" width="20.09765625" customWidth="1"/>
-    <col min="5" max="5" width="21.296875" customWidth="1"/>
-    <col min="6" max="6" width="10.796875" customWidth="1"/>
-    <col min="7" max="7" width="11.3984375" customWidth="1"/>
-    <col min="8" max="8" width="12.59765625" customWidth="1"/>
-    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="5" max="6" width="21.296875" customWidth="1"/>
+    <col min="7" max="7" width="10.796875" customWidth="1"/>
+    <col min="8" max="8" width="11.3984375" customWidth="1"/>
+    <col min="9" max="9" width="12.59765625" customWidth="1"/>
+    <col min="10" max="10" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
@@ -697,873 +712,969 @@
         <v>6</v>
       </c>
       <c r="F2" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="J2" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B3" s="3">
         <v>45076</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="4">
+      <c r="H3" s="4">
         <v>4500</v>
       </c>
-      <c r="H3" s="4">
+      <c r="I3" s="4">
         <v>598</v>
       </c>
-      <c r="I3" s="5">
-        <f>H3/G3</f>
+      <c r="J3" s="5">
+        <f>I3/H3</f>
         <v>0.13288888888888889</v>
       </c>
     </row>
-    <row r="4" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B4" s="3">
         <v>45076</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="4">
+      <c r="H4" s="4">
         <v>3800</v>
       </c>
-      <c r="H4" s="4">
+      <c r="I4" s="4">
         <v>1045</v>
       </c>
-      <c r="I4" s="5">
-        <f t="shared" ref="I4:I32" si="0">H4/G4</f>
+      <c r="J4" s="5">
+        <f t="shared" ref="J4:J32" si="0">I4/H4</f>
         <v>0.27500000000000002</v>
       </c>
     </row>
-    <row r="5" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B5" s="3">
         <v>45076</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="4">
+        <v>70</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="4">
         <v>3712.5</v>
       </c>
-      <c r="H5" s="4">
+      <c r="I5" s="4">
         <v>1009</v>
       </c>
-      <c r="I5" s="5">
+      <c r="J5" s="5">
         <f t="shared" si="0"/>
         <v>0.2717845117845118</v>
       </c>
     </row>
-    <row r="6" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B6" s="3">
         <v>45076</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4">
+        <v>72</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4">
         <v>779</v>
       </c>
-      <c r="I6" s="5" t="e">
+      <c r="J6" s="5" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="7" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B7" s="3">
         <v>45076</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="4">
+      <c r="H7" s="4">
         <v>5000</v>
       </c>
-      <c r="H7" s="4">
+      <c r="I7" s="4">
         <v>684</v>
       </c>
-      <c r="I7" s="5">
+      <c r="J7" s="5">
         <f t="shared" si="0"/>
         <v>0.1368</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B8" s="3">
         <v>45077</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="4">
+      <c r="H8" s="4">
         <v>6100</v>
       </c>
-      <c r="H8" s="4">
+      <c r="I8" s="4">
         <v>544</v>
       </c>
-      <c r="I8" s="5">
+      <c r="J8" s="5">
         <f t="shared" si="0"/>
         <v>8.9180327868852466E-2</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B9" s="3">
         <v>45077</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F9" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="4">
+      <c r="H9" s="4">
         <v>4625</v>
       </c>
-      <c r="H9" s="4">
+      <c r="I9" s="4">
         <v>670</v>
       </c>
-      <c r="I9" s="5">
+      <c r="J9" s="5">
         <f t="shared" si="0"/>
         <v>0.14486486486486486</v>
       </c>
     </row>
-    <row r="10" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>45077</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="4">
+      <c r="H10" s="4">
         <v>3800</v>
       </c>
-      <c r="H10" s="4">
+      <c r="I10" s="4">
         <v>2045</v>
       </c>
-      <c r="I10" s="5">
+      <c r="J10" s="5">
         <f t="shared" si="0"/>
         <v>0.53815789473684206</v>
       </c>
     </row>
-    <row r="11" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <v>45077</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="4">
+      <c r="H11" s="4">
         <v>3600</v>
       </c>
-      <c r="H11" s="4">
+      <c r="I11" s="4">
         <v>1564</v>
       </c>
-      <c r="I11" s="5">
+      <c r="J11" s="5">
         <f t="shared" si="0"/>
         <v>0.43444444444444447</v>
       </c>
     </row>
-    <row r="12" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
         <v>45077</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F12" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="4">
+      <c r="H12" s="4">
         <v>5100</v>
       </c>
-      <c r="H12" s="4">
+      <c r="I12" s="4">
         <v>1220</v>
       </c>
-      <c r="I12" s="5">
+      <c r="J12" s="5">
         <f t="shared" si="0"/>
         <v>0.23921568627450981</v>
       </c>
     </row>
-    <row r="13" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B13" s="3">
         <v>45077</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G13" s="4">
+      <c r="H13" s="4">
         <v>4750</v>
       </c>
-      <c r="H13" s="4">
+      <c r="I13" s="4">
         <v>1435</v>
       </c>
-      <c r="I13" s="5">
+      <c r="J13" s="5">
         <f t="shared" si="0"/>
         <v>0.30210526315789471</v>
       </c>
     </row>
-    <row r="14" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
         <v>45077</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="F14" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G14" s="4">
+      <c r="H14" s="4">
         <v>6000</v>
       </c>
-      <c r="H14" s="4">
+      <c r="I14" s="4">
         <v>998</v>
       </c>
-      <c r="I14" s="5">
+      <c r="J14" s="5">
         <f t="shared" si="0"/>
         <v>0.16633333333333333</v>
       </c>
     </row>
-    <row r="15" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B15" s="3">
         <v>45077</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="F15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G15" s="4">
+      <c r="H15" s="4">
         <v>4500</v>
       </c>
-      <c r="H15" s="4">
+      <c r="I15" s="4">
         <v>780</v>
       </c>
-      <c r="I15" s="5">
+      <c r="J15" s="5">
         <f t="shared" si="0"/>
         <v>0.17333333333333334</v>
       </c>
     </row>
-    <row r="16" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <v>45078</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="F16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4">
+      <c r="H16" s="4"/>
+      <c r="I16" s="4">
         <v>1044</v>
       </c>
-      <c r="I16" s="5" t="e">
+      <c r="J16" s="5" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B17" s="3">
         <v>45078</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="F17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G17" s="4">
+      <c r="H17" s="4">
         <v>3712.5</v>
       </c>
-      <c r="H17" s="4">
+      <c r="I17" s="4">
         <v>1222</v>
       </c>
-      <c r="I17" s="5">
+      <c r="J17" s="5">
         <f t="shared" si="0"/>
         <v>0.32915824915824915</v>
       </c>
     </row>
-    <row r="18" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B18" s="3">
         <v>45078</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="F18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G18" s="4">
+      <c r="H18" s="4">
         <v>4950</v>
       </c>
-      <c r="H18" s="4">
+      <c r="I18" s="4">
         <v>1065</v>
       </c>
-      <c r="I18" s="5">
+      <c r="J18" s="5">
         <f t="shared" si="0"/>
         <v>0.21515151515151515</v>
       </c>
     </row>
-    <row r="19" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B19" s="3">
         <v>45078</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="F19" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G19" s="4">
+      <c r="H19" s="4">
         <v>4750</v>
       </c>
-      <c r="H19" s="4">
+      <c r="I19" s="4">
         <v>810</v>
       </c>
-      <c r="I19" s="5">
+      <c r="J19" s="5">
         <f t="shared" si="0"/>
         <v>0.17052631578947369</v>
       </c>
     </row>
-    <row r="20" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B20" s="3">
         <v>45078</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="F20" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G20" s="4">
+      <c r="H20" s="4">
         <v>7320</v>
       </c>
-      <c r="H20" s="4">
+      <c r="I20" s="4">
         <v>933</v>
       </c>
-      <c r="I20" s="5">
+      <c r="J20" s="5">
         <f t="shared" si="0"/>
         <v>0.12745901639344262</v>
       </c>
     </row>
-    <row r="21" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B21" s="3">
         <v>45077</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="F21" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G21" s="4">
+      <c r="H21" s="4">
         <v>6000</v>
       </c>
-      <c r="H21" s="4">
+      <c r="I21" s="4">
         <v>998</v>
       </c>
-      <c r="I21" s="5">
-        <f t="shared" ref="I21:I22" si="1">H21/G21</f>
+      <c r="J21" s="5">
+        <f t="shared" ref="J21:J22" si="1">I21/H21</f>
         <v>0.16633333333333333</v>
       </c>
     </row>
-    <row r="22" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B22" s="3">
         <v>45077</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="F22" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G22" s="4">
+      <c r="H22" s="4">
         <v>4500</v>
       </c>
-      <c r="H22" s="4">
+      <c r="I22" s="4">
         <v>780</v>
       </c>
-      <c r="I22" s="5">
+      <c r="J22" s="5">
         <f t="shared" si="1"/>
         <v>0.17333333333333334</v>
       </c>
     </row>
-    <row r="23" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B23" s="3">
         <v>45078</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="F23" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G23" s="4">
+      <c r="H23" s="4">
         <v>5087.5</v>
       </c>
-      <c r="H23" s="4">
+      <c r="I23" s="4">
         <v>655</v>
       </c>
-      <c r="I23" s="5">
+      <c r="J23" s="5">
         <f t="shared" si="0"/>
         <v>0.12874692874692875</v>
       </c>
     </row>
-    <row r="24" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B24" s="3">
         <v>45078</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="F24" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G24" s="4">
+      <c r="H24" s="4">
         <v>4500</v>
       </c>
-      <c r="H24" s="4">
+      <c r="I24" s="4">
         <v>722</v>
       </c>
-      <c r="I24" s="5">
+      <c r="J24" s="5">
         <f t="shared" si="0"/>
         <v>0.16044444444444445</v>
       </c>
     </row>
-    <row r="25" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B25" s="3">
         <v>45078</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="F25" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G25" s="4">
+      <c r="H25" s="4">
         <v>4250</v>
       </c>
-      <c r="H25" s="4">
+      <c r="I25" s="4">
         <v>901</v>
       </c>
-      <c r="I25" s="5">
+      <c r="J25" s="5">
         <f t="shared" si="0"/>
         <v>0.21199999999999999</v>
       </c>
     </row>
-    <row r="26" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B26" s="3">
         <v>45079</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="F26" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G26" s="4">
+      <c r="H26" s="4">
         <v>5250</v>
       </c>
-      <c r="H26" s="4">
+      <c r="I26" s="4">
         <v>1349</v>
       </c>
-      <c r="I26" s="5">
+      <c r="J26" s="5">
         <f t="shared" si="0"/>
         <v>0.25695238095238093</v>
       </c>
     </row>
-    <row r="27" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B27" s="3">
         <v>45079</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="F27" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G27" s="4">
+      <c r="H27" s="4">
         <v>6500</v>
       </c>
-      <c r="H27" s="4">
+      <c r="I27" s="4">
         <v>1288</v>
       </c>
-      <c r="I27" s="5">
+      <c r="J27" s="5">
         <f t="shared" si="0"/>
         <v>0.19815384615384615</v>
       </c>
     </row>
-    <row r="28" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B28" s="3">
         <v>45079</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="F28" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G28" s="4">
+      <c r="H28" s="4">
         <v>7500</v>
       </c>
-      <c r="H28" s="4">
+      <c r="I28" s="4">
         <v>1664</v>
       </c>
-      <c r="I28" s="5">
+      <c r="J28" s="5">
         <f t="shared" si="0"/>
         <v>0.22186666666666666</v>
       </c>
     </row>
-    <row r="29" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B29" s="3">
         <v>45079</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="F29" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G29" s="4">
+      <c r="H29" s="4">
         <v>5500</v>
       </c>
-      <c r="H29" s="4">
+      <c r="I29" s="4">
         <v>1320</v>
       </c>
-      <c r="I29" s="5">
+      <c r="J29" s="5">
         <f t="shared" si="0"/>
         <v>0.24</v>
       </c>
     </row>
-    <row r="30" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B30" s="3">
         <v>45079</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D30" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="F30" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G30" s="4">
+      <c r="H30" s="4">
         <v>4625</v>
       </c>
-      <c r="H30" s="4">
+      <c r="I30" s="4">
         <v>1001</v>
       </c>
-      <c r="I30" s="5">
+      <c r="J30" s="5">
         <f t="shared" si="0"/>
         <v>0.21643243243243243</v>
       </c>
     </row>
-    <row r="31" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B31" s="3">
         <v>45079</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D31" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F31" s="2" t="s">
+      <c r="G31" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G31" s="4">
+      <c r="H31" s="4">
         <v>4500</v>
       </c>
-      <c r="H31" s="4">
+      <c r="I31" s="4">
         <v>960</v>
       </c>
-      <c r="I31" s="5">
+      <c r="J31" s="5">
         <f t="shared" si="0"/>
         <v>0.21333333333333335</v>
       </c>
     </row>
-    <row r="32" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B32" s="3">
         <v>45079</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="F32" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G32" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G32" s="4">
+      <c r="H32" s="4">
         <v>5400</v>
       </c>
-      <c r="H32" s="4">
+      <c r="I32" s="4">
         <v>540</v>
       </c>
-      <c r="I32" s="5">
+      <c r="J32" s="5">
         <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
     </row>
-    <row r="33" spans="2:9" ht="18" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:10" ht="18" x14ac:dyDescent="0.3">
       <c r="B33" s="3">
         <v>45076</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="F33" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G33" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G33" s="4">
+      <c r="H33" s="4">
         <v>5000</v>
       </c>
-      <c r="H33" s="4">
+      <c r="I33" s="4">
         <v>684</v>
       </c>
-      <c r="I33" s="5">
-        <f t="shared" ref="I33" si="2">H33/G33</f>
+      <c r="J33" s="5">
+        <f t="shared" ref="J33" si="2">I33/H33</f>
         <v>0.1368</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G34" s="1"/>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G35" s="1"/>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G36" s="1"/>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G37" s="1"/>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G38" s="1"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G39" s="1"/>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G40" s="1"/>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G41" s="1"/>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G42" s="1"/>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H34" s="1"/>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H35" s="1"/>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H36" s="1"/>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H37" s="1"/>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H38" s="1"/>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H39" s="1"/>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H40" s="1"/>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H41" s="1"/>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="H42" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Blank Cells are replaced with N/A
</commit_message>
<xml_diff>
--- a/Day 4/Data Cleaning Start.xlsx
+++ b/Day 4/Data Cleaning Start.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20058B7-D13C-41CD-9028-CE77F77F9C90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C0DD881-01BE-4ED0-A28D-A78EA04B3912}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{7F7E1DDE-3781-814A-825E-072C922D74F6}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="78">
   <si>
     <t>Date</t>
   </si>
@@ -266,6 +266,9 @@
   </si>
   <si>
     <t>State</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -803,7 +806,9 @@
       <c r="F5" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="G5" s="2"/>
+      <c r="G5" s="2" t="s">
+        <v>77</v>
+      </c>
       <c r="H5" s="4">
         <v>3712.5</v>
       </c>
@@ -831,14 +836,18 @@
       <c r="F6" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="4"/>
+      <c r="G6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>77</v>
+      </c>
       <c r="I6" s="4">
         <v>779</v>
       </c>
       <c r="J6" s="5" t="e">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="7" spans="2:10" ht="18" x14ac:dyDescent="0.3">
@@ -1130,13 +1139,15 @@
       <c r="G16" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="4"/>
+      <c r="H16" s="4" t="s">
+        <v>77</v>
+      </c>
       <c r="I16" s="4">
         <v>1044</v>
       </c>
       <c r="J16" s="5" t="e">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="17" spans="2:10" ht="18" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Errors showing for Profit Margin are replaced with N/A
</commit_message>
<xml_diff>
--- a/Day 4/Data Cleaning Start.xlsx
+++ b/Day 4/Data Cleaning Start.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C0DD881-01BE-4ED0-A28D-A78EA04B3912}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE8B50B1-DC99-4D77-9A3D-0594865970CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{7F7E1DDE-3781-814A-825E-072C922D74F6}"/>
   </bookViews>
@@ -756,7 +756,7 @@
         <v>598</v>
       </c>
       <c r="J3" s="5">
-        <f>I3/H3</f>
+        <f>IFERROR(I3/H3,"N/A")</f>
         <v>0.13288888888888889</v>
       </c>
     </row>
@@ -786,7 +786,7 @@
         <v>1045</v>
       </c>
       <c r="J4" s="5">
-        <f t="shared" ref="J4:J32" si="0">I4/H4</f>
+        <f t="shared" ref="J4:J33" si="0">IFERROR(I4/H4,"N/A")</f>
         <v>0.27500000000000002</v>
       </c>
     </row>
@@ -845,9 +845,9 @@
       <c r="I6" s="4">
         <v>779</v>
       </c>
-      <c r="J6" s="5" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+      <c r="J6" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>N/A</v>
       </c>
     </row>
     <row r="7" spans="2:10" ht="18" x14ac:dyDescent="0.3">
@@ -1145,9 +1145,9 @@
       <c r="I16" s="4">
         <v>1044</v>
       </c>
-      <c r="J16" s="5" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+      <c r="J16" s="5" t="str">
+        <f t="shared" si="0"/>
+        <v>N/A</v>
       </c>
     </row>
     <row r="17" spans="2:10" ht="18" x14ac:dyDescent="0.3">
@@ -1296,7 +1296,7 @@
         <v>998</v>
       </c>
       <c r="J21" s="5">
-        <f t="shared" ref="J21:J22" si="1">I21/H21</f>
+        <f t="shared" si="0"/>
         <v>0.16633333333333333</v>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
         <v>780</v>
       </c>
       <c r="J22" s="5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.17333333333333334</v>
       </c>
     </row>
@@ -1656,7 +1656,7 @@
         <v>684</v>
       </c>
       <c r="J33" s="5">
-        <f t="shared" ref="J33" si="2">I33/H33</f>
+        <f t="shared" si="0"/>
         <v>0.1368</v>
       </c>
     </row>

</xml_diff>